<commit_message>
Patch#54: Added Pagination to Products - Added Pagination to Products - Added Cache Service and Cache Manager - Added UX when Permisison is denied - Fix Restore and Backup Feature - Added UX for Transaction to scroll down when input detail transaction - Added Unit when Editing Transaction - When Updating, Pressing Enter will Trigger Update - Added UX for Up Arrow in Purchasing - Added Feature to Import Categories and Supplier at the same time - Fix Unit in Master Stock to be Uppercase - Added README
</commit_message>
<xml_diff>
--- a/testing_files/products/test_products_200_rows.xlsx
+++ b/testing_files/products/test_products_200_rows.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Program\POS PyQt6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Program\POS PyQt6\testing_files\products\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44F5AF2-22DA-43F3-A5A2-93F5A7EE095A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49538A8-4600-47B1-9FD4-AD8015AD8DD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17172" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="542">
   <si>
     <t>SKU</t>
   </si>
@@ -1552,6 +1552,105 @@
   </si>
   <si>
     <t>SKU007</t>
+  </si>
+  <si>
+    <t>Automotive</t>
+  </si>
+  <si>
+    <t>Global Traders</t>
+  </si>
+  <si>
+    <t>Pet Supplies</t>
+  </si>
+  <si>
+    <t>Style Outfitters</t>
+  </si>
+  <si>
+    <t>Food &amp; Beverage</t>
+  </si>
+  <si>
+    <t>I-Store</t>
+  </si>
+  <si>
+    <t>Health &amp; Beauty</t>
+  </si>
+  <si>
+    <t>The Home Store</t>
+  </si>
+  <si>
+    <t>Jewelry &amp; Watches</t>
+  </si>
+  <si>
+    <t>Easy Living</t>
+  </si>
+  <si>
+    <t>Furniture</t>
+  </si>
+  <si>
+    <t>Home Essentials</t>
+  </si>
+  <si>
+    <t>Style &amp; More</t>
+  </si>
+  <si>
+    <t>Toys &amp; Games</t>
+  </si>
+  <si>
+    <t>Perfect Home</t>
+  </si>
+  <si>
+    <t>Care Products Ltd</t>
+  </si>
+  <si>
+    <t>Stationery</t>
+  </si>
+  <si>
+    <t>Baby &amp; Child</t>
+  </si>
+  <si>
+    <t>Eco Supplies</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Fresh Imports</t>
+  </si>
+  <si>
+    <t>Prime Distributors</t>
+  </si>
+  <si>
+    <t>U-Store</t>
+  </si>
+  <si>
+    <t>Tech Innovators</t>
+  </si>
+  <si>
+    <t>Clothing</t>
+  </si>
+  <si>
+    <t>Home Supplies</t>
+  </si>
+  <si>
+    <t>Bargain Box</t>
+  </si>
+  <si>
+    <t>Garden &amp; Outdoor</t>
+  </si>
+  <si>
+    <t>Beauty &amp; Personal Care</t>
+  </si>
+  <si>
+    <t>All Seasons</t>
+  </si>
+  <si>
+    <t>Office Supplies</t>
+  </si>
+  <si>
+    <t>Art &amp; Crafts</t>
+  </si>
+  <si>
+    <t>Personal Care</t>
   </si>
 </sst>
 </file>
@@ -1715,10 +1814,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1744,7 +1843,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1769,8 +1868,14 @@
       <c r="H2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I2" t="s">
+        <v>509</v>
+      </c>
+      <c r="J2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1795,8 +1900,14 @@
       <c r="H3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I3" t="s">
+        <v>511</v>
+      </c>
+      <c r="J3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1815,8 +1926,14 @@
       <c r="G4">
         <v>95</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I4" t="s">
+        <v>513</v>
+      </c>
+      <c r="J4" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>508</v>
       </c>
@@ -1838,8 +1955,14 @@
       <c r="G5">
         <v>87</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5" t="s">
+        <v>515</v>
+      </c>
+      <c r="J5" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1858,8 +1981,14 @@
       <c r="G6">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I6" t="s">
+        <v>517</v>
+      </c>
+      <c r="J6" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1878,8 +2007,14 @@
       <c r="G7">
         <v>54</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I7" t="s">
+        <v>519</v>
+      </c>
+      <c r="J7" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1901,8 +2036,14 @@
       <c r="H8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I8" t="s">
+        <v>511</v>
+      </c>
+      <c r="J8" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -1921,8 +2062,14 @@
       <c r="G9">
         <v>88</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I9" t="s">
+        <v>522</v>
+      </c>
+      <c r="J9" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -1944,8 +2091,14 @@
       <c r="G10">
         <v>87</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I10" t="s">
+        <v>519</v>
+      </c>
+      <c r="J10" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1961,8 +2114,14 @@
       <c r="G11">
         <v>99</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I11" t="s">
+        <v>525</v>
+      </c>
+      <c r="J11" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>36</v>
       </c>
@@ -1987,8 +2146,14 @@
       <c r="H12" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I12" t="s">
+        <v>526</v>
+      </c>
+      <c r="J12" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -2010,8 +2175,14 @@
       <c r="H13" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I13" t="s">
+        <v>528</v>
+      </c>
+      <c r="J13" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -2036,8 +2207,14 @@
       <c r="H14" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I14" t="s">
+        <v>517</v>
+      </c>
+      <c r="J14" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>50</v>
       </c>
@@ -2062,8 +2239,14 @@
       <c r="H15" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I15" t="s">
+        <v>513</v>
+      </c>
+      <c r="J15" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>55</v>
       </c>
@@ -2085,8 +2268,14 @@
       <c r="H16" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I16" t="s">
+        <v>515</v>
+      </c>
+      <c r="J16" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -2108,8 +2297,14 @@
       <c r="H17" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I17" t="s">
+        <v>511</v>
+      </c>
+      <c r="J17" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>62</v>
       </c>
@@ -2134,8 +2329,14 @@
       <c r="H18" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I18" t="s">
+        <v>513</v>
+      </c>
+      <c r="J18" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -2160,8 +2361,14 @@
       <c r="H19" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I19" t="s">
+        <v>528</v>
+      </c>
+      <c r="J19" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -2183,8 +2390,14 @@
       <c r="H20" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I20" t="s">
+        <v>509</v>
+      </c>
+      <c r="J20" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -2209,8 +2422,14 @@
       <c r="H21" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I21" t="s">
+        <v>511</v>
+      </c>
+      <c r="J21" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -2229,8 +2448,14 @@
       <c r="G22">
         <v>96</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I22" t="s">
+        <v>517</v>
+      </c>
+      <c r="J22" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>79</v>
       </c>
@@ -2255,8 +2480,14 @@
       <c r="H23" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I23" t="s">
+        <v>517</v>
+      </c>
+      <c r="J23" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>82</v>
       </c>
@@ -2281,8 +2512,14 @@
       <c r="H24" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I24" t="s">
+        <v>533</v>
+      </c>
+      <c r="J24" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>86</v>
       </c>
@@ -2304,8 +2541,14 @@
       <c r="H25" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I25" t="s">
+        <v>528</v>
+      </c>
+      <c r="J25" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>89</v>
       </c>
@@ -2327,8 +2570,14 @@
       <c r="G26">
         <v>234</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I26" t="s">
+        <v>534</v>
+      </c>
+      <c r="J26" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>93</v>
       </c>
@@ -2350,8 +2599,14 @@
       <c r="H27" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I27" t="s">
+        <v>526</v>
+      </c>
+      <c r="J27" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>96</v>
       </c>
@@ -2373,8 +2628,14 @@
       <c r="G28">
         <v>403</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I28" t="s">
+        <v>519</v>
+      </c>
+      <c r="J28" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>99</v>
       </c>
@@ -2399,8 +2660,14 @@
       <c r="H29" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I29" t="s">
+        <v>519</v>
+      </c>
+      <c r="J29" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>103</v>
       </c>
@@ -2425,8 +2692,14 @@
       <c r="H30" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I30" t="s">
+        <v>515</v>
+      </c>
+      <c r="J30" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>105</v>
       </c>
@@ -2448,8 +2721,14 @@
       <c r="H31" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I31" t="s">
+        <v>513</v>
+      </c>
+      <c r="J31" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>108</v>
       </c>
@@ -2474,8 +2753,14 @@
       <c r="H32" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I32" t="s">
+        <v>536</v>
+      </c>
+      <c r="J32" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>110</v>
       </c>
@@ -2500,8 +2785,14 @@
       <c r="H33" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I33" t="s">
+        <v>519</v>
+      </c>
+      <c r="J33" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>113</v>
       </c>
@@ -2526,8 +2817,14 @@
       <c r="H34" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I34" t="s">
+        <v>537</v>
+      </c>
+      <c r="J34" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>116</v>
       </c>
@@ -2549,8 +2846,14 @@
       <c r="H35" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I35" t="s">
+        <v>511</v>
+      </c>
+      <c r="J35" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>119</v>
       </c>
@@ -2572,8 +2875,14 @@
       <c r="H36" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I36" t="s">
+        <v>537</v>
+      </c>
+      <c r="J36" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>121</v>
       </c>
@@ -2595,8 +2904,14 @@
       <c r="H37" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I37" t="s">
+        <v>511</v>
+      </c>
+      <c r="J37" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>123</v>
       </c>
@@ -2618,8 +2933,14 @@
       <c r="H38" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I38" t="s">
+        <v>528</v>
+      </c>
+      <c r="J38" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>125</v>
       </c>
@@ -2641,8 +2962,14 @@
       <c r="H39" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I39" t="s">
+        <v>522</v>
+      </c>
+      <c r="J39" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>128</v>
       </c>
@@ -2667,8 +2994,14 @@
       <c r="H40" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I40" t="s">
+        <v>519</v>
+      </c>
+      <c r="J40" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>131</v>
       </c>
@@ -2690,8 +3023,14 @@
       <c r="H41" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I41" t="s">
+        <v>539</v>
+      </c>
+      <c r="J41" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>133</v>
       </c>
@@ -2716,8 +3055,14 @@
       <c r="H42" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I42" t="s">
+        <v>525</v>
+      </c>
+      <c r="J42" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>136</v>
       </c>
@@ -2742,8 +3087,14 @@
       <c r="H43" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I43" t="s">
+        <v>528</v>
+      </c>
+      <c r="J43" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>138</v>
       </c>
@@ -2765,8 +3116,14 @@
       <c r="G44">
         <v>441</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I44" t="s">
+        <v>526</v>
+      </c>
+      <c r="J44" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>141</v>
       </c>
@@ -2791,8 +3148,14 @@
       <c r="H45" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I45" t="s">
+        <v>511</v>
+      </c>
+      <c r="J45" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>144</v>
       </c>
@@ -2817,8 +3180,14 @@
       <c r="H46" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I46" t="s">
+        <v>522</v>
+      </c>
+      <c r="J46" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>147</v>
       </c>
@@ -2843,8 +3212,14 @@
       <c r="H47" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I47" t="s">
+        <v>534</v>
+      </c>
+      <c r="J47" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>150</v>
       </c>
@@ -2869,8 +3244,14 @@
       <c r="H48" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I48" t="s">
+        <v>509</v>
+      </c>
+      <c r="J48" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>152</v>
       </c>
@@ -2892,8 +3273,14 @@
       <c r="H49" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I49" t="s">
+        <v>522</v>
+      </c>
+      <c r="J49" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>155</v>
       </c>
@@ -2915,8 +3302,14 @@
       <c r="H50" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I50" t="s">
+        <v>525</v>
+      </c>
+      <c r="J50" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>157</v>
       </c>
@@ -2938,8 +3331,14 @@
       <c r="H51" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I51" t="s">
+        <v>540</v>
+      </c>
+      <c r="J51" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>160</v>
       </c>
@@ -2961,8 +3360,14 @@
       <c r="H52" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I52" t="s">
+        <v>541</v>
+      </c>
+      <c r="J52" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>162</v>
       </c>
@@ -2984,8 +3389,14 @@
       <c r="H53" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I53" t="s">
+        <v>513</v>
+      </c>
+      <c r="J53" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>165</v>
       </c>
@@ -3010,8 +3421,14 @@
       <c r="H54" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I54" t="s">
+        <v>534</v>
+      </c>
+      <c r="J54" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>167</v>
       </c>
@@ -3036,8 +3453,14 @@
       <c r="H55" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I55" t="s">
+        <v>539</v>
+      </c>
+      <c r="J55" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>170</v>
       </c>
@@ -3062,8 +3485,14 @@
       <c r="H56" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I56" t="s">
+        <v>513</v>
+      </c>
+      <c r="J56" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>173</v>
       </c>
@@ -3088,8 +3517,14 @@
       <c r="H57" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I57" t="s">
+        <v>537</v>
+      </c>
+      <c r="J57" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>176</v>
       </c>
@@ -3108,8 +3543,14 @@
       <c r="G58">
         <v>225</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I58" t="s">
+        <v>541</v>
+      </c>
+      <c r="J58" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>179</v>
       </c>
@@ -3134,8 +3575,14 @@
       <c r="H59" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I59" t="s">
+        <v>539</v>
+      </c>
+      <c r="J59" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>181</v>
       </c>
@@ -3160,8 +3607,14 @@
       <c r="H60" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I60" t="s">
+        <v>536</v>
+      </c>
+      <c r="J60" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>183</v>
       </c>
@@ -3183,8 +3636,14 @@
       <c r="H61" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I61" t="s">
+        <v>533</v>
+      </c>
+      <c r="J61" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>186</v>
       </c>
@@ -3206,8 +3665,14 @@
       <c r="H62" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I62" t="s">
+        <v>515</v>
+      </c>
+      <c r="J62" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>188</v>
       </c>
@@ -3232,8 +3697,14 @@
       <c r="H63" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I63" t="s">
+        <v>515</v>
+      </c>
+      <c r="J63" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>190</v>
       </c>
@@ -3252,8 +3723,14 @@
       <c r="G64">
         <v>445</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I64" t="s">
+        <v>525</v>
+      </c>
+      <c r="J64" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>193</v>
       </c>
@@ -3278,8 +3755,14 @@
       <c r="H65" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I65" t="s">
+        <v>533</v>
+      </c>
+      <c r="J65" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>196</v>
       </c>
@@ -3301,8 +3784,14 @@
       <c r="H66" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I66" t="s">
+        <v>528</v>
+      </c>
+      <c r="J66" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>199</v>
       </c>
@@ -3324,8 +3813,14 @@
       <c r="H67" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I67" t="s">
+        <v>537</v>
+      </c>
+      <c r="J67" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>202</v>
       </c>
@@ -3350,8 +3845,14 @@
       <c r="H68" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I68" t="s">
+        <v>534</v>
+      </c>
+      <c r="J68" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>205</v>
       </c>
@@ -3376,8 +3877,14 @@
       <c r="H69" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I69" t="s">
+        <v>519</v>
+      </c>
+      <c r="J69" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>207</v>
       </c>
@@ -3402,8 +3909,14 @@
       <c r="H70" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I70" t="s">
+        <v>539</v>
+      </c>
+      <c r="J70" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>210</v>
       </c>
@@ -3428,8 +3941,14 @@
       <c r="H71" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I71" t="s">
+        <v>517</v>
+      </c>
+      <c r="J71" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>213</v>
       </c>
@@ -3451,8 +3970,14 @@
       <c r="H72" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I72" t="s">
+        <v>541</v>
+      </c>
+      <c r="J72" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>215</v>
       </c>
@@ -3474,8 +3999,14 @@
       <c r="H73" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I73" t="s">
+        <v>534</v>
+      </c>
+      <c r="J73" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>217</v>
       </c>
@@ -3497,8 +4028,14 @@
       <c r="H74" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I74" t="s">
+        <v>539</v>
+      </c>
+      <c r="J74" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>219</v>
       </c>
@@ -3520,8 +4057,14 @@
       <c r="H75" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I75" t="s">
+        <v>519</v>
+      </c>
+      <c r="J75" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>221</v>
       </c>
@@ -3543,8 +4086,14 @@
       <c r="H76" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I76" t="s">
+        <v>533</v>
+      </c>
+      <c r="J76" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>223</v>
       </c>
@@ -3569,8 +4118,14 @@
       <c r="H77" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I77" t="s">
+        <v>526</v>
+      </c>
+      <c r="J77" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>226</v>
       </c>
@@ -3595,8 +4150,14 @@
       <c r="H78" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I78" t="s">
+        <v>534</v>
+      </c>
+      <c r="J78" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>229</v>
       </c>
@@ -3621,8 +4182,14 @@
       <c r="H79" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I79" t="s">
+        <v>528</v>
+      </c>
+      <c r="J79" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>232</v>
       </c>
@@ -3647,8 +4214,14 @@
       <c r="H80" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I80" t="s">
+        <v>522</v>
+      </c>
+      <c r="J80" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>234</v>
       </c>
@@ -3673,8 +4246,14 @@
       <c r="H81" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I81" t="s">
+        <v>537</v>
+      </c>
+      <c r="J81" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>237</v>
       </c>
@@ -3696,8 +4275,14 @@
       <c r="H82" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I82" t="s">
+        <v>541</v>
+      </c>
+      <c r="J82" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>239</v>
       </c>
@@ -3719,8 +4304,14 @@
       <c r="H83" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I83" t="s">
+        <v>522</v>
+      </c>
+      <c r="J83" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>241</v>
       </c>
@@ -3742,8 +4333,14 @@
       <c r="H84" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="85" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I84" t="s">
+        <v>515</v>
+      </c>
+      <c r="J84" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>244</v>
       </c>
@@ -3765,8 +4362,14 @@
       <c r="H85" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I85" t="s">
+        <v>534</v>
+      </c>
+      <c r="J85" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>246</v>
       </c>
@@ -3791,8 +4394,14 @@
       <c r="H86" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="87" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I86" t="s">
+        <v>536</v>
+      </c>
+      <c r="J86" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>248</v>
       </c>
@@ -3814,8 +4423,14 @@
       <c r="H87" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I87" t="s">
+        <v>540</v>
+      </c>
+      <c r="J87" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>250</v>
       </c>
@@ -3837,8 +4452,14 @@
       <c r="H88" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="89" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I88" t="s">
+        <v>537</v>
+      </c>
+      <c r="J88" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>252</v>
       </c>
@@ -3863,8 +4484,14 @@
       <c r="H89" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I89" t="s">
+        <v>522</v>
+      </c>
+      <c r="J89" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>254</v>
       </c>
@@ -3886,8 +4513,14 @@
       <c r="H90" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I90" t="s">
+        <v>540</v>
+      </c>
+      <c r="J90" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>257</v>
       </c>
@@ -3909,8 +4542,14 @@
       <c r="H91" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I91" t="s">
+        <v>513</v>
+      </c>
+      <c r="J91" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>260</v>
       </c>
@@ -3935,8 +4574,14 @@
       <c r="H92" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I92" t="s">
+        <v>528</v>
+      </c>
+      <c r="J92" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>262</v>
       </c>
@@ -3958,8 +4603,14 @@
       <c r="G93">
         <v>251</v>
       </c>
-    </row>
-    <row r="94" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I93" t="s">
+        <v>522</v>
+      </c>
+      <c r="J93" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>265</v>
       </c>
@@ -3984,8 +4635,14 @@
       <c r="H94" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="95" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I94" t="s">
+        <v>534</v>
+      </c>
+      <c r="J94" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>268</v>
       </c>
@@ -4007,8 +4664,14 @@
       <c r="H95" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="96" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I95" t="s">
+        <v>517</v>
+      </c>
+      <c r="J95" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>271</v>
       </c>
@@ -4030,8 +4693,14 @@
       <c r="G96">
         <v>388</v>
       </c>
-    </row>
-    <row r="97" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I96" t="s">
+        <v>541</v>
+      </c>
+      <c r="J96" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>273</v>
       </c>
@@ -4053,8 +4722,14 @@
       <c r="H97" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="98" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I97" t="s">
+        <v>533</v>
+      </c>
+      <c r="J97" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>276</v>
       </c>
@@ -4076,8 +4751,14 @@
       <c r="H98" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="99" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I98" t="s">
+        <v>533</v>
+      </c>
+      <c r="J98" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>278</v>
       </c>
@@ -4099,8 +4780,14 @@
       <c r="H99" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="100" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I99" t="s">
+        <v>528</v>
+      </c>
+      <c r="J99" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>280</v>
       </c>
@@ -4125,8 +4812,14 @@
       <c r="H100" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="101" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I100" t="s">
+        <v>540</v>
+      </c>
+      <c r="J100" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>282</v>
       </c>
@@ -4148,8 +4841,14 @@
       <c r="G101">
         <v>262</v>
       </c>
-    </row>
-    <row r="102" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I101" t="s">
+        <v>537</v>
+      </c>
+      <c r="J101" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>284</v>
       </c>
@@ -4174,8 +4873,14 @@
       <c r="H102" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="103" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I102" t="s">
+        <v>533</v>
+      </c>
+      <c r="J102" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>286</v>
       </c>
@@ -4200,8 +4905,14 @@
       <c r="H103" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="104" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I103" t="s">
+        <v>515</v>
+      </c>
+      <c r="J103" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>289</v>
       </c>
@@ -4226,8 +4937,14 @@
       <c r="H104" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="105" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I104" t="s">
+        <v>534</v>
+      </c>
+      <c r="J104" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>292</v>
       </c>
@@ -4249,8 +4966,14 @@
       <c r="G105">
         <v>473</v>
       </c>
-    </row>
-    <row r="106" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I105" t="s">
+        <v>537</v>
+      </c>
+      <c r="J105" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>295</v>
       </c>
@@ -4272,8 +4995,14 @@
       <c r="H106" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="107" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I106" t="s">
+        <v>541</v>
+      </c>
+      <c r="J106" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>297</v>
       </c>
@@ -4298,8 +5027,14 @@
       <c r="H107" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="108" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I107" t="s">
+        <v>525</v>
+      </c>
+      <c r="J107" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>299</v>
       </c>
@@ -4321,8 +5056,14 @@
       <c r="H108" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="109" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I108" t="s">
+        <v>513</v>
+      </c>
+      <c r="J108" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>301</v>
       </c>
@@ -4347,8 +5088,14 @@
       <c r="H109" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="110" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I109" t="s">
+        <v>537</v>
+      </c>
+      <c r="J109" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>303</v>
       </c>
@@ -4370,8 +5117,14 @@
       <c r="H110" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="111" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I110" t="s">
+        <v>528</v>
+      </c>
+      <c r="J110" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>305</v>
       </c>
@@ -4396,8 +5149,14 @@
       <c r="H111" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="112" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I111" t="s">
+        <v>511</v>
+      </c>
+      <c r="J111" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>307</v>
       </c>
@@ -4419,8 +5178,14 @@
       <c r="H112" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="113" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I112" t="s">
+        <v>509</v>
+      </c>
+      <c r="J112" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>309</v>
       </c>
@@ -4445,8 +5210,14 @@
       <c r="H113" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="114" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I113" t="s">
+        <v>537</v>
+      </c>
+      <c r="J113" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>312</v>
       </c>
@@ -4471,8 +5242,14 @@
       <c r="H114" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="115" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I114" t="s">
+        <v>522</v>
+      </c>
+      <c r="J114" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>315</v>
       </c>
@@ -4497,8 +5274,14 @@
       <c r="H115" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="116" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I115" t="s">
+        <v>513</v>
+      </c>
+      <c r="J115" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>317</v>
       </c>
@@ -4520,8 +5303,14 @@
       <c r="H116" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="117" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I116" t="s">
+        <v>511</v>
+      </c>
+      <c r="J116" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>319</v>
       </c>
@@ -4546,8 +5335,14 @@
       <c r="H117" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="118" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I117" t="s">
+        <v>519</v>
+      </c>
+      <c r="J117" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>321</v>
       </c>
@@ -4569,8 +5364,14 @@
       <c r="H118" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="119" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I118" t="s">
+        <v>536</v>
+      </c>
+      <c r="J118" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>324</v>
       </c>
@@ -4595,8 +5396,14 @@
       <c r="H119" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="120" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I119" t="s">
+        <v>509</v>
+      </c>
+      <c r="J119" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>326</v>
       </c>
@@ -4621,8 +5428,14 @@
       <c r="H120" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="121" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I120" t="s">
+        <v>540</v>
+      </c>
+      <c r="J120" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>328</v>
       </c>
@@ -4647,8 +5460,14 @@
       <c r="H121" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="122" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I121" t="s">
+        <v>515</v>
+      </c>
+      <c r="J121" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>330</v>
       </c>
@@ -4670,8 +5489,14 @@
       <c r="G122">
         <v>101</v>
       </c>
-    </row>
-    <row r="123" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I122" t="s">
+        <v>511</v>
+      </c>
+      <c r="J122" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>332</v>
       </c>
@@ -4693,8 +5518,14 @@
       <c r="H123" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="124" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I123" t="s">
+        <v>509</v>
+      </c>
+      <c r="J123" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>334</v>
       </c>
@@ -4716,8 +5547,14 @@
       <c r="H124" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="125" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I124" t="s">
+        <v>525</v>
+      </c>
+      <c r="J124" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>336</v>
       </c>
@@ -4739,8 +5576,14 @@
       <c r="H125" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="126" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I125" t="s">
+        <v>519</v>
+      </c>
+      <c r="J125" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>338</v>
       </c>
@@ -4762,8 +5605,14 @@
       <c r="H126" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="127" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I126" t="s">
+        <v>509</v>
+      </c>
+      <c r="J126" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>340</v>
       </c>
@@ -4785,8 +5634,14 @@
       <c r="H127" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="128" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I127" t="s">
+        <v>517</v>
+      </c>
+      <c r="J127" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>343</v>
       </c>
@@ -4805,8 +5660,14 @@
       <c r="G128">
         <v>326</v>
       </c>
-    </row>
-    <row r="129" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I128" t="s">
+        <v>519</v>
+      </c>
+      <c r="J128" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>346</v>
       </c>
@@ -4831,8 +5692,14 @@
       <c r="H129" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="130" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I129" t="s">
+        <v>533</v>
+      </c>
+      <c r="J129" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>348</v>
       </c>
@@ -4857,8 +5724,14 @@
       <c r="H130" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="131" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I130" t="s">
+        <v>533</v>
+      </c>
+      <c r="J130" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>351</v>
       </c>
@@ -4883,8 +5756,14 @@
       <c r="H131" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="132" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I131" t="s">
+        <v>511</v>
+      </c>
+      <c r="J131" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>353</v>
       </c>
@@ -4909,8 +5788,14 @@
       <c r="H132" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="133" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I132" t="s">
+        <v>537</v>
+      </c>
+      <c r="J132" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>355</v>
       </c>
@@ -4932,8 +5817,14 @@
       <c r="H133" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="134" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I133" t="s">
+        <v>525</v>
+      </c>
+      <c r="J133" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>357</v>
       </c>
@@ -4955,8 +5846,14 @@
       <c r="H134" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="135" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I134" t="s">
+        <v>536</v>
+      </c>
+      <c r="J134" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>359</v>
       </c>
@@ -4981,8 +5878,14 @@
       <c r="H135" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="136" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I135" t="s">
+        <v>541</v>
+      </c>
+      <c r="J135" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>361</v>
       </c>
@@ -5004,8 +5907,14 @@
       <c r="H136" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="137" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I136" t="s">
+        <v>539</v>
+      </c>
+      <c r="J136" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>364</v>
       </c>
@@ -5027,8 +5936,14 @@
       <c r="H137" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="138" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I137" t="s">
+        <v>526</v>
+      </c>
+      <c r="J137" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>366</v>
       </c>
@@ -5053,8 +5968,14 @@
       <c r="H138" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="139" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I138" t="s">
+        <v>522</v>
+      </c>
+      <c r="J138" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>368</v>
       </c>
@@ -5079,8 +6000,14 @@
       <c r="H139" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="140" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I139" t="s">
+        <v>522</v>
+      </c>
+      <c r="J139" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>371</v>
       </c>
@@ -5105,8 +6032,14 @@
       <c r="H140" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="141" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I140" t="s">
+        <v>536</v>
+      </c>
+      <c r="J140" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>373</v>
       </c>
@@ -5128,8 +6061,14 @@
       <c r="H141" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="142" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I141" t="s">
+        <v>541</v>
+      </c>
+      <c r="J141" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>375</v>
       </c>
@@ -5154,8 +6093,14 @@
       <c r="H142" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="143" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I142" t="s">
+        <v>534</v>
+      </c>
+      <c r="J142" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>377</v>
       </c>
@@ -5180,8 +6125,14 @@
       <c r="H143" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="144" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I143" t="s">
+        <v>525</v>
+      </c>
+      <c r="J143" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>379</v>
       </c>
@@ -5203,8 +6154,14 @@
       <c r="G144">
         <v>420</v>
       </c>
-    </row>
-    <row r="145" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I144" t="s">
+        <v>526</v>
+      </c>
+      <c r="J144" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>381</v>
       </c>
@@ -5223,8 +6180,14 @@
       <c r="G145">
         <v>59</v>
       </c>
-    </row>
-    <row r="146" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I145" t="s">
+        <v>525</v>
+      </c>
+      <c r="J145" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>383</v>
       </c>
@@ -5243,8 +6206,14 @@
       <c r="G146">
         <v>404</v>
       </c>
-    </row>
-    <row r="147" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I146" t="s">
+        <v>509</v>
+      </c>
+      <c r="J146" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>386</v>
       </c>
@@ -5269,8 +6238,14 @@
       <c r="H147" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="148" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I147" t="s">
+        <v>522</v>
+      </c>
+      <c r="J147" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>388</v>
       </c>
@@ -5289,8 +6264,14 @@
       <c r="G148">
         <v>295</v>
       </c>
-    </row>
-    <row r="149" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I148" t="s">
+        <v>536</v>
+      </c>
+      <c r="J148" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>390</v>
       </c>
@@ -5312,8 +6293,14 @@
       <c r="H149" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="150" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I149" t="s">
+        <v>539</v>
+      </c>
+      <c r="J149" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>393</v>
       </c>
@@ -5335,8 +6322,14 @@
       <c r="H150" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="151" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I150" t="s">
+        <v>539</v>
+      </c>
+      <c r="J150" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>395</v>
       </c>
@@ -5361,8 +6354,14 @@
       <c r="H151" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="152" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I151" t="s">
+        <v>522</v>
+      </c>
+      <c r="J151" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>397</v>
       </c>
@@ -5381,8 +6380,14 @@
       <c r="G152">
         <v>168</v>
       </c>
-    </row>
-    <row r="153" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I152" t="s">
+        <v>515</v>
+      </c>
+      <c r="J152" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>399</v>
       </c>
@@ -5404,8 +6409,14 @@
       <c r="H153" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="154" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I153" t="s">
+        <v>513</v>
+      </c>
+      <c r="J153" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>402</v>
       </c>
@@ -5427,8 +6438,14 @@
       <c r="H154" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="155" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I154" t="s">
+        <v>517</v>
+      </c>
+      <c r="J154" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>404</v>
       </c>
@@ -5453,8 +6470,14 @@
       <c r="H155" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="156" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I155" t="s">
+        <v>533</v>
+      </c>
+      <c r="J155" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>406</v>
       </c>
@@ -5476,8 +6499,14 @@
       <c r="H156" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="157" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I156" t="s">
+        <v>536</v>
+      </c>
+      <c r="J156" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>408</v>
       </c>
@@ -5499,8 +6528,14 @@
       <c r="H157" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="158" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I157" t="s">
+        <v>534</v>
+      </c>
+      <c r="J157" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>411</v>
       </c>
@@ -5522,8 +6557,14 @@
       <c r="G158">
         <v>446</v>
       </c>
-    </row>
-    <row r="159" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I158" t="s">
+        <v>537</v>
+      </c>
+      <c r="J158" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>413</v>
       </c>
@@ -5545,8 +6586,14 @@
       <c r="H159" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="160" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I159" t="s">
+        <v>515</v>
+      </c>
+      <c r="J159" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>415</v>
       </c>
@@ -5565,8 +6612,14 @@
       <c r="G160">
         <v>398</v>
       </c>
-    </row>
-    <row r="161" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I160" t="s">
+        <v>540</v>
+      </c>
+      <c r="J160" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>417</v>
       </c>
@@ -5588,8 +6641,14 @@
       <c r="G161">
         <v>485</v>
       </c>
-    </row>
-    <row r="162" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I161" t="s">
+        <v>509</v>
+      </c>
+      <c r="J161" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>419</v>
       </c>
@@ -5611,8 +6670,14 @@
       <c r="H162" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="163" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I162" t="s">
+        <v>515</v>
+      </c>
+      <c r="J162" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>421</v>
       </c>
@@ -5634,8 +6699,14 @@
       <c r="H163" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="164" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I163" t="s">
+        <v>511</v>
+      </c>
+      <c r="J163" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>423</v>
       </c>
@@ -5657,8 +6728,14 @@
       <c r="H164" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="165" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I164" t="s">
+        <v>522</v>
+      </c>
+      <c r="J164" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="165" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>425</v>
       </c>
@@ -5680,8 +6757,14 @@
       <c r="H165" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="166" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I165" t="s">
+        <v>539</v>
+      </c>
+      <c r="J165" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="166" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>428</v>
       </c>
@@ -5703,8 +6786,14 @@
       <c r="H166" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="167" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I166" t="s">
+        <v>528</v>
+      </c>
+      <c r="J166" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>430</v>
       </c>
@@ -5726,8 +6815,14 @@
       <c r="H167" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="168" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I167" t="s">
+        <v>540</v>
+      </c>
+      <c r="J167" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>433</v>
       </c>
@@ -5752,8 +6847,14 @@
       <c r="H168" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="169" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I168" t="s">
+        <v>515</v>
+      </c>
+      <c r="J168" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>435</v>
       </c>
@@ -5778,8 +6879,14 @@
       <c r="H169" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="170" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I169" t="s">
+        <v>513</v>
+      </c>
+      <c r="J169" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>437</v>
       </c>
@@ -5801,8 +6908,14 @@
       <c r="H170" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="171" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I170" t="s">
+        <v>519</v>
+      </c>
+      <c r="J170" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>440</v>
       </c>
@@ -5824,8 +6937,14 @@
       <c r="H171" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="172" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I171" t="s">
+        <v>522</v>
+      </c>
+      <c r="J171" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>442</v>
       </c>
@@ -5847,8 +6966,14 @@
       <c r="H172" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="173" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I172" t="s">
+        <v>526</v>
+      </c>
+      <c r="J172" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>445</v>
       </c>
@@ -5870,8 +6995,14 @@
       <c r="H173" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="174" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I173" t="s">
+        <v>537</v>
+      </c>
+      <c r="J173" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>447</v>
       </c>
@@ -5893,8 +7024,14 @@
       <c r="H174" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="175" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I174" t="s">
+        <v>511</v>
+      </c>
+      <c r="J174" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>449</v>
       </c>
@@ -5916,8 +7053,14 @@
       <c r="H175" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="176" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I175" t="s">
+        <v>533</v>
+      </c>
+      <c r="J175" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>451</v>
       </c>
@@ -5942,8 +7085,14 @@
       <c r="H176" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="177" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I176" t="s">
+        <v>515</v>
+      </c>
+      <c r="J176" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>453</v>
       </c>
@@ -5965,8 +7114,14 @@
       <c r="H177" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="178" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I177" t="s">
+        <v>517</v>
+      </c>
+      <c r="J177" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="178" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>455</v>
       </c>
@@ -5988,8 +7143,14 @@
       <c r="H178" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="179" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I178" t="s">
+        <v>526</v>
+      </c>
+      <c r="J178" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>457</v>
       </c>
@@ -6011,8 +7172,14 @@
       <c r="H179" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="180" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I179" t="s">
+        <v>539</v>
+      </c>
+      <c r="J179" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="180" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>459</v>
       </c>
@@ -6037,8 +7204,14 @@
       <c r="H180" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="181" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I180" t="s">
+        <v>534</v>
+      </c>
+      <c r="J180" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="181" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>462</v>
       </c>
@@ -6060,8 +7233,14 @@
       <c r="H181" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="182" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I181" t="s">
+        <v>534</v>
+      </c>
+      <c r="J181" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="182" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>464</v>
       </c>
@@ -6080,8 +7259,14 @@
       <c r="G182">
         <v>320</v>
       </c>
-    </row>
-    <row r="183" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I182" t="s">
+        <v>537</v>
+      </c>
+      <c r="J182" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="183" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>466</v>
       </c>
@@ -6103,8 +7288,14 @@
       <c r="H183" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="184" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I183" t="s">
+        <v>534</v>
+      </c>
+      <c r="J183" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="184" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>468</v>
       </c>
@@ -6123,8 +7314,14 @@
       <c r="G184">
         <v>128</v>
       </c>
-    </row>
-    <row r="185" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I184" t="s">
+        <v>515</v>
+      </c>
+      <c r="J184" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="185" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>471</v>
       </c>
@@ -6146,8 +7343,14 @@
       <c r="H185" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="186" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I185" t="s">
+        <v>515</v>
+      </c>
+      <c r="J185" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="186" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>473</v>
       </c>
@@ -6169,8 +7372,14 @@
       <c r="H186" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="187" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I186" t="s">
+        <v>515</v>
+      </c>
+      <c r="J186" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>475</v>
       </c>
@@ -6195,8 +7404,14 @@
       <c r="H187" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="188" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I187" t="s">
+        <v>519</v>
+      </c>
+      <c r="J187" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="188" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>477</v>
       </c>
@@ -6218,8 +7433,14 @@
       <c r="H188" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="189" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I188" t="s">
+        <v>526</v>
+      </c>
+      <c r="J188" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="189" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>479</v>
       </c>
@@ -6244,8 +7465,14 @@
       <c r="H189" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="190" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I189" t="s">
+        <v>540</v>
+      </c>
+      <c r="J189" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="190" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>482</v>
       </c>
@@ -6270,8 +7497,14 @@
       <c r="H190" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="191" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I190" t="s">
+        <v>517</v>
+      </c>
+      <c r="J190" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="191" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>484</v>
       </c>
@@ -6293,8 +7526,14 @@
       <c r="H191" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="192" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I191" t="s">
+        <v>519</v>
+      </c>
+      <c r="J191" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>486</v>
       </c>
@@ -6313,8 +7552,14 @@
       <c r="G192">
         <v>459</v>
       </c>
-    </row>
-    <row r="193" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I192" t="s">
+        <v>537</v>
+      </c>
+      <c r="J192" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="193" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>488</v>
       </c>
@@ -6339,8 +7584,14 @@
       <c r="H193" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="194" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I193" t="s">
+        <v>525</v>
+      </c>
+      <c r="J193" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="194" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>491</v>
       </c>
@@ -6362,8 +7613,14 @@
       <c r="H194" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="195" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I194" t="s">
+        <v>517</v>
+      </c>
+      <c r="J194" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="195" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>493</v>
       </c>
@@ -6385,8 +7642,14 @@
       <c r="H195" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="196" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I195" t="s">
+        <v>519</v>
+      </c>
+      <c r="J195" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="196" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>495</v>
       </c>
@@ -6408,8 +7671,14 @@
       <c r="H196" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="197" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I196" t="s">
+        <v>515</v>
+      </c>
+      <c r="J196" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>497</v>
       </c>
@@ -6431,8 +7700,14 @@
       <c r="H197" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="198" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I197" t="s">
+        <v>539</v>
+      </c>
+      <c r="J197" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="198" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>499</v>
       </c>
@@ -6457,8 +7732,14 @@
       <c r="H198" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="199" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I198" t="s">
+        <v>525</v>
+      </c>
+      <c r="J198" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="199" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>501</v>
       </c>
@@ -6477,8 +7758,14 @@
       <c r="G199">
         <v>68</v>
       </c>
-    </row>
-    <row r="200" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I199" t="s">
+        <v>534</v>
+      </c>
+      <c r="J199" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="200" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>503</v>
       </c>
@@ -6500,8 +7787,14 @@
       <c r="H200" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="201" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I200" t="s">
+        <v>513</v>
+      </c>
+      <c r="J200" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="201" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>506</v>
       </c>
@@ -6525,6 +7818,12 @@
       </c>
       <c r="H201" t="s">
         <v>68</v>
+      </c>
+      <c r="I201" t="s">
+        <v>536</v>
+      </c>
+      <c r="J201" t="s">
+        <v>535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>